<commit_message>
updated to use macroarea group intercept
</commit_message>
<xml_diff>
--- a/output/Table_A_Consensus.xlsx
+++ b/output/Table_A_Consensus.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E61"/>
+  <dimension ref="A1:E60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -472,7 +472,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>4.870569298366846</v>
+        <v>4.835146850686929</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -483,21 +483,21 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1611ka</t>
+          <t>0179bka</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>verb-patient agreement &gt; verb-agent agreement</t>
+          <t>gender Dem &gt; number Dem</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>All languages with verb-patient agreement, regardless of type, also have verb agreement with the agent as well.</t>
+          <t>There is a hierarchy: Number &gt; Gender &gt; Case, such that if some target agrees in one category on the hierarchy then it will also agree in all categories higher on the hierarchy.</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>2.934815213719705</v>
+        <v>4.664502587297177</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -508,21 +508,21 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0045ka</t>
+          <t>0564ka</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Obj indexing &gt; Sbj indexing</t>
+          <t>Du (noun) &gt; Du (pronoun)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>If there is a construction in which the verb agrees with some member of the relational hierarchy Subject &gt; DO &gt; IO &gt; Oblique &gt; [Genitive], then there are at least some constructions in which the verb agrees with members higher on that hierarchy .</t>
+          <t>If the Dual extends to nouns, it also extends to pronouns.</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>2.936821197335671</v>
+        <v>4.054680264358921</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -533,21 +533,21 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1053ka</t>
+          <t>0179aka</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>agreement determiners &gt; agreement modifiers</t>
+          <t>gender Adj &gt; number Adj</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>If determiners agree within NPs, modifiers are likelier also to agree than not to agree.</t>
+          <t>There is a hierarchy: Number &gt; Gender &gt; Case, such that if some target agrees in one category on the hierarchy then it will also agree in all categories higher on the hierarchy.</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1.870688030367973</v>
+        <v>4.112830766047429</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -572,7 +572,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>3.36518311257479</v>
+        <v>3.513355905301345</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -583,21 +583,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0179cka</t>
+          <t>0045ka</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>gender Art &gt; number Art</t>
+          <t>Obj indexing &gt; Sbj indexing</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>There is a hierarchy: Number &gt; Gender &gt; Case, such that if some target agrees in one category on the hierarchy then it will also agree in all categories higher on the hierarchy.</t>
+          <t>If there is a construction in which the verb agrees with some member of the relational hierarchy Subject &gt; DO &gt; IO &gt; Oblique &gt; [Genitive], then there are at least some constructions in which the verb agrees with members higher on that hierarchy .</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>19.99893669886151</v>
+        <v>3.246506350419219</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -608,21 +608,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0179bka</t>
+          <t>1611ka</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>gender Dem &gt; number Dem</t>
+          <t>verb-patient agreement &gt; verb-agent agreement</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>There is a hierarchy: Number &gt; Gender &gt; Case, such that if some target agrees in one category on the hierarchy then it will also agree in all categories higher on the hierarchy.</t>
+          <t>All languages with verb-patient agreement, regardless of type, also have verb agreement with the agent as well.</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>4.23734651520502</v>
+        <v>3.243084761453067</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -647,7 +647,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>2.440244954998791</v>
+        <v>2.646038367650203</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -658,21 +658,21 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0179aka</t>
+          <t>0328ka</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>gender Adj &gt; number Adj</t>
+          <t>verb agr S prefix &gt; verb agr P</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>There is a hierarchy: Number &gt; Gender &gt; Case, such that if some target agrees in one category on the hierarchy then it will also agree in all categories higher on the hierarchy.</t>
+          <t>If a verb agrees with a subject in prefix, then verbs have affixes or clitics which agree with the direct object.</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>4.016055512377319</v>
+        <v>2.754290172141838</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -683,21 +683,21 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0328ka</t>
+          <t>0320ka</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>verb agr S prefix &gt; verb agr P</t>
+          <t>nom/acc pronouns &gt; nom/acc nouns</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>If a verb agrees with a subject in prefix, then verbs have affixes or clitics which agree with the direct object.</t>
+          <t>If personal pronouns have an opposition of the syntactic forms of nominative and accusative, then this opposition is relevant for nouns as well.</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>2.492324303553454</v>
+        <v>3.173729281049036</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -708,21 +708,21 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0320ka</t>
+          <t>1053ka</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>nom/acc pronouns &gt; nom/acc nouns</t>
+          <t>agreement determiners &gt; agreement modifiers</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>If personal pronouns have an opposition of the syntactic forms of nominative and accusative, then this opposition is relevant for nouns as well.</t>
+          <t>If determiners agree within NPs, modifiers are likelier also to agree than not to agree.</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>2.62083459091826</v>
+        <v>1.928720792784927</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -733,21 +733,21 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>1163ka</t>
+          <t>0084ka</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>indefinite article &gt; definite article</t>
+          <t>verb agreement &gt; agreement S</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>If a language has a grammaticalized indefinite article, it is likely to also have a definite article, while the reverse does not necessarily hold true.</t>
+          <t>If in a language the verb agrees with anything, it agrees with some or all subjects.</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>2.054681397622355</v>
+        <v>2.374152595412502</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -758,21 +758,21 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0564ka</t>
+          <t>0057aka</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Du (noun) &gt; Du (pronoun)</t>
+          <t>Adj-N &gt; Num-N</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>If the Dual extends to nouns, it also extends to pronouns.</t>
+          <t>Universal 18. When the descriptive adjective precedes the noun, the demonstrative and the numeral, with overwhelmingly more than chance frequency, do likewise.</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>3.050901338920796</v>
+        <v>2.266875056421193</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -797,7 +797,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>1.816828793215298</v>
+        <v>1.831776760822278</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -808,21 +808,21 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0084ka</t>
+          <t>0073ka</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>verb agreement &gt; agreement S</t>
+          <t>N-Dem &gt; N-Adj</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>If in a language the verb agrees with anything, it agrees with some or all subjects.</t>
+          <t>If the demonstrative determiner follows the noun, then the adjective follows the noun.</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>2.112774285456635</v>
+        <v>1.794825975181644</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -833,21 +833,21 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0332ka</t>
+          <t>0489ka</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>o suffix &gt; s suffix</t>
+          <t>SOV &gt; N-Adp</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>If the suffix position is the only possible one for an object-affix,  then the subject-affix also occupies this position at least in some  cases.</t>
+          <t>Universal 4. With overwhelmingly greater than chance frequency, languages with normal SOV order are postpositional.</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>2.123020607493848</v>
+        <v>2.328404573988429</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -858,21 +858,21 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0073ka</t>
+          <t>1163ka</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>N-Dem &gt; N-Adj</t>
+          <t>indefinite article &gt; definite article</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>If the demonstrative determiner follows the noun, then the adjective follows the noun.</t>
+          <t>If a language has a grammaticalized indefinite article, it is likely to also have a definite article, while the reverse does not necessarily hold true.</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>1.768017971374062</v>
+        <v>1.939264098820795</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -883,21 +883,21 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0237aka</t>
+          <t>0075ka</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>number Adj &gt; number noun</t>
+          <t>N-Num &gt; N-Adj</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>If adjectives inflect for any category, nouns inflect for this category as well.</t>
+          <t>If a language has noun before numeral, then it has noun before adjective.</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>1.599004674038305</v>
+        <v>2.390911383782132</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -908,21 +908,21 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0057aka</t>
+          <t>0331bka</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Adj-N &gt; Num-N</t>
+          <t>s prefix &gt; o prefix | o suffix (weak)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Universal 18. When the descriptive adjective precedes the noun, the demonstrative and the numeral, with overwhelmingly more than chance frequency, do likewise.</t>
+          <t>If the prefix position is the only possible one for a subject-affix, then  the object-affix also occupies this position in all forms (with the  exception of Wolio) or at least in some of them (no exceptions).</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>2.30803383416191</v>
+        <v>2.764781653216753</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -933,21 +933,21 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0276ka</t>
+          <t>0332ka</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>number (adjective | verb) &gt; number (noun)</t>
+          <t>o suffix &gt; s suffix</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>If there is a regular number distinction in the forms of the adjective or of the verb, there is the same distinction in the forms of the noun of  the given language.</t>
+          <t>If the suffix position is the only possible one for an object-affix,  then the subject-affix also occupies this position at least in some  cases.</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>1.579756084098748</v>
+        <v>2.55111460638247</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -958,21 +958,21 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0075ka</t>
+          <t>0511bka</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>N-Num &gt; N-Adj</t>
+          <t>Dual &gt; Plural</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>If a language has noun before numeral, then it has noun before adjective.</t>
+          <t>Universal 34. No language has a trial number unless it has a dual. No language has a dual unless it has a plural.</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>2.292839847410399</v>
+        <v>3.340474473362873</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -983,21 +983,21 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0489ka</t>
+          <t>0177ka</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>SOV &gt; N-Adp</t>
+          <t>N-Adp &amp; Dem-N &gt; Gen-N</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Universal 4. With overwhelmingly greater than chance frequency, languages with normal SOV order are postpositional.</t>
+          <t>If a language has Postp word order, then if the demonstrative precedes the noun, the genitive precedes the noun.</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>2.419895521433984</v>
+        <v>2.064822224675335</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -1008,21 +1008,21 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>0331bka</t>
+          <t>0166ka</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>s prefix &gt; o prefix | o suffix (weak)</t>
+          <t>pref-V Obj &gt; V Agr Sbj</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>If the prefix position is the only possible one for a subject-affix, then  the object-affix also occupies this position in all forms (with the  exception of Wolio) or at least in some of them (no exceptions).</t>
+          <t>If a verb agrees in prefix with the direct object, then at least some of the verbs agree with the subject.</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>2.446184392276208</v>
+        <v>2.838238256330807</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -1033,21 +1033,21 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>0511bka</t>
+          <t>0237aka</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Dual &gt; Plural</t>
+          <t>number Adj &gt; number noun</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Universal 34. No language has a trial number unless it has a dual. No language has a dual unless it has a plural.</t>
+          <t>If adjectives inflect for any category, nouns inflect for this category as well.</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>3.692141249324536</v>
+        <v>1.61363604402148</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -1072,7 +1072,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>-2.217746553261749</v>
+        <v>-2.132657677811546</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -1083,21 +1083,21 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>0177ka</t>
+          <t>0276ka</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>N-Adp &amp; Dem-N &gt; Gen-N</t>
+          <t>number (adjective | verb) &gt; number (noun)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>If a language has Postp word order, then if the demonstrative precedes the noun, the genitive precedes the noun.</t>
+          <t>If there is a regular number distinction in the forms of the adjective or of the verb, there is the same distinction in the forms of the noun of  the given language.</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>1.992677597512943</v>
+        <v>1.562093203714124</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1108,21 +1108,21 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>0057bka</t>
+          <t>0179cka</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Adj-N &gt; Dem-N</t>
+          <t>gender Art &gt; number Art</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Universal 18. When the descriptive adjective precedes the noun, the demonstrative and the numeral, with overwhelmingly more than chance frequency, do likewise.</t>
+          <t>There is a hierarchy: Number &gt; Gender &gt; Case, such that if some target agrees in one category on the hierarchy then it will also agree in all categories higher on the hierarchy.</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>1.743367890158452</v>
+        <v>48.25501405811831</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1147,7 +1147,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>1.858677136659366</v>
+        <v>1.976350924271603</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1158,21 +1158,21 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>1415ka</t>
+          <t>0001_or_2aka</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>poss agree &gt; verbal agree S</t>
+          <t>Adp-N &gt; N-Gen</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>If heads of possessive constructions agree with their possessors in a given language then verbs agree with subjects in that language. Standardized IF heads of possessive constructions (=possessees) agree with their possessors, THEN verbs agree with subjects.</t>
+          <t>Universal 2. In languages with prepositions, the genitive almost always follows the governing noun, while in languages with postpositions it almost always precedes</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>1.341792939127774</v>
+        <v>2.031864658657858</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1183,21 +1183,21 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>0238aka</t>
+          <t>0093ka</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>rigid order &gt; SV</t>
+          <t>gender 2SG &gt; gender 3SG</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>If constituent order is rigid, all determined constituents precede their respective determining constituents; in particular, subjects precede their predicates, verbs their complements (objects, prepositional phrases), prepositions their complements (noun phrases), head nouns their attributive adjectives, relative clauses, and complements (prepositional phrases).</t>
+          <t>IF a language has pronominal gender in the 2nd person singular, THEN it has a greater probability of having this distinction in the 3rd person singular than of not having it.</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>1.19231960667703</v>
+        <v>10.06150184375314</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1208,21 +1208,21 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>0166ka</t>
+          <t>0238aka</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>pref-V Obj &gt; V Agr Sbj</t>
+          <t>rigid order &gt; SV</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>If a verb agrees in prefix with the direct object, then at least some of the verbs agree with the subject.</t>
+          <t>If constituent order is rigid, all determined constituents precede their respective determining constituents; in particular, subjects precede their predicates, verbs their complements (objects, prepositional phrases), prepositions their complements (noun phrases), head nouns their attributive adjectives, relative clauses, and complements (prepositional phrases).</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>2.863955955921274</v>
+        <v>1.216022151960379</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1233,21 +1233,21 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>0001_or_2aka</t>
+          <t>0057bka</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Adp-N &gt; N-Gen</t>
+          <t>Adj-N &gt; Dem-N</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Universal 2. In languages with prepositions, the genitive almost always follows the governing noun, while in languages with postpositions it almost always precedes</t>
+          <t>Universal 18. When the descriptive adjective precedes the noun, the demonstrative and the numeral, with overwhelmingly more than chance frequency, do likewise.</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>1.952871649950399</v>
+        <v>1.589261195617346</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1258,21 +1258,21 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>0096ka</t>
+          <t>1267bka</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>N-Adp &amp; (Adj-N | Rel-N) &gt; PossPron-N</t>
+          <t>SVO &gt; not ergative</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>IF there are postpositions, THEN (IF adjectives precede nouns or relatives precede nouns, THEN demonstratives preced nouns and numerals precede nouns and possessives preced nouns) and (IF demonstratives precede nouns or numerals precede nouns or possessives precede nouns, THEN genitives precede nouns).</t>
+          <t>Ergative systems are found only in SOV and VSO languages. SVO languages are never ergative.</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>1.797907515282995</v>
+        <v>2.116341755267067</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1283,21 +1283,21 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>0446ka</t>
+          <t>1415ka</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>V-final | free &gt; N-Adp | case</t>
+          <t>poss agree &gt; verbal agree S</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>If a language has Verb-final (rigid, or non-rigid) or free word order as (one of) its basic word order(s), then it has postpositions or case affixes.</t>
+          <t>If heads of possessive constructions agree with their possessors in a given language then verbs agree with subjects in that language. Standardized IF heads of possessive constructions (=possessees) agree with their possessors, THEN verbs agree with subjects.</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>1.20414038174528</v>
+        <v>1.488538464378867</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1308,21 +1308,21 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>0230bka</t>
+          <t>0446ka</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>no case &gt; Adp-N</t>
+          <t>V-final | free &gt; N-Adp | case</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>IF constituent order is rigid, THEN cases are absent, and vice versa; ; If cases are absent, THEN the use of prepositions is extensive, and vice versa;; IF order is rigid, THEN the use of prepositions is extensive, and vice versa. : IF constituent order is flexible, THEN cases are present, and vice versa; ; IF cases are present, THEN the use of prepositions is sparse, and vice versa; ; IF order is flexible, THEN the use of prepositions is sparse, and vice versa.</t>
+          <t>If a language has Verb-final (rigid, or non-rigid) or free word order as (one of) its basic word order(s), then it has postpositions or case affixes.</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>1.138783026135591</v>
+        <v>1.48360726519953</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1333,21 +1333,21 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>1741ka</t>
+          <t>0096ka</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Gen prefix &gt; verbal prefixes</t>
+          <t>N-Adp &amp; (Adj-N | Rel-N) &gt; PossPron-N</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>There is more prefixing on verb than on noun. If a language has any prefixes on noun, it will also have prefixes on verb with considerably more than chance frequency.</t>
+          <t>IF there are postpositions, THEN (IF adjectives precede nouns or relatives precede nouns, THEN demonstratives preced nouns and numerals precede nouns and possessives preced nouns) and (IF demonstratives precede nouns or numerals precede nouns or possessives precede nouns, THEN genitives precede nouns).</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>1.386353980377046</v>
+        <v>1.715558302531373</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1358,21 +1358,21 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>0072ka</t>
+          <t>0612ka</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Adp-N &amp; N-Dem &gt; N-Adj</t>
+          <t>switch-reference marking &gt; V-final</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>If a language has Prep word order, then if the demonstrative determiner follows the noun, the adjective follows the noun.</t>
+          <t>If there is Switch-Reference marking, languages will mostly be verb-final.</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>1.317031861308654</v>
+        <v>1.58121596554337</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1383,21 +1383,21 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>1267bka</t>
+          <t>0173ka</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>SVO &gt; not ergative</t>
+          <t>Adp-N &amp; N-Dem &gt; N-Gen</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Ergative systems are found only in SOV and VSO languages. SVO languages are never ergative.</t>
+          <t>If a language is prepositional, then if the demonstrative follows the noun, the genitive follows the noun.</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>2.059675732407101</v>
+        <v>1.526834691935651</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1408,21 +1408,21 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>0069ka</t>
+          <t>0230eka</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Adp-N &amp; N-Adj &gt; N-Gen</t>
+          <t>case &gt; no Adp-N</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>If a language has Prep word order, then if the adjective follows the noun, the genitive follows the noun.</t>
+          <t>IF constituent order is rigid, THEN cases are absent, and vice versa; ; If cases are absent, THEN the use of prepositions is extensive, and vice versa;; IF order is rigid, THEN the use of prepositions is extensive, and vice versa. : IF constituent order is flexible, THEN cases are present, and vice versa; ; IF cases are present, THEN the use of prepositions is sparse, and vice versa; ; IF order is flexible, THEN the use of prepositions is sparse, and vice versa.</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>1.241144762883292</v>
+        <v>1.356345570617479</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1433,21 +1433,21 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>0612ka</t>
+          <t>0069ka</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>switch-reference marking &gt; V-final</t>
+          <t>Adp-N &amp; N-Adj &gt; N-Gen</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>If there is Switch-Reference marking, languages will mostly be verb-final.</t>
+          <t>If a language has Prep word order, then if the adjective follows the noun, the genitive follows the noun.</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>1.61338287848973</v>
+        <v>1.418384605190932</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1458,21 +1458,21 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>0093ka</t>
+          <t>0095aka</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>gender 2SG &gt; gender 3SG</t>
+          <t>N-Adp &amp; (Adj-N | Rel-N) &gt; Dem-N</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>IF a language has pronominal gender in the 2nd person singular, THEN it has a greater probability of having this distinction in the 3rd person singular than of not having it.</t>
+          <t>IF there are postpositions, THEN (IF adjectives precede nouns or relatives precede nouns, THEN demonstratives preced nouns and numerals precede nouns) and (IF demonstratives precede nouns or numerals precede nouns, THEN genitives precede nouns).</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>9.921878118556819</v>
+        <v>1.457470580768031</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1483,21 +1483,21 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>1586ka</t>
+          <t>0015aka</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>poss head-marked &gt; opp alien-inalien poss</t>
+          <t>OV &gt; V-Mod</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>An opposition of "alienable" and "inalienable" possession is almost inevitable in languages where possession is regularly head-marked. The alienable-inalienable opposition is almost never signaled by dependent-marked morphology.</t>
+          <t>Verbal modifiers like those for negation, causation, and reflexive or reciprocal are placed after verb roots in OV languages and before verb roots in VO languages.</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>1.020138745543415</v>
+        <v>1.354844463380237</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1508,21 +1508,21 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>1027cka</t>
+          <t>0072ka</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>no case &gt; no morph tense | VO</t>
+          <t>Adp-N &amp; N-Dem &gt; N-Adj</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>There are correlations between following parameters: VO word order, Non-tensedness, Non-casedness, WITH-Construction, Non-Absolute Converb. Standardized IF VO, THEN Non-tensedness, Non-casedness, WITH-Construction, and Non-Absolute Converb. IF Non-tensedness, THEN VO, Non-casedness, WITH-Construction, and Non-Absolute Converb. IF Non-casedness, THEN VO, Non-tensedness, WITH-Construction, and Non-Absolute Converb. IF AND-construction, THEN VO, Non-tensedness, Non-casedness, and Non-Absolute Converb. IF Non-Absolute Converb, THEN VO, Non-tensedness, Non-casedness, and WITH-Construction.</t>
+          <t>If a language has Prep word order, then if the demonstrative determiner follows the noun, the adjective follows the noun.</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>1.142291476016037</v>
+        <v>1.289252994691377</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1533,21 +1533,21 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>0173ka</t>
+          <t>0074ka</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Adp-N &amp; N-Dem &gt; N-Gen</t>
+          <t>Adp-N &amp; N-Num &gt; N-Adj</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>If a language is prepositional, then if the demonstrative follows the noun, the genitive follows the noun.</t>
+          <t>If a language has Prep word order, then if the numeral follows the noun, the adjective follows the noun.</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>1.130273129131531</v>
+        <v>1.610968746684149</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1558,21 +1558,21 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>0230eka</t>
+          <t>1027cka</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>case &gt; no Adp-N</t>
+          <t>no case &gt; no morph tense | VO</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>IF constituent order is rigid, THEN cases are absent, and vice versa; ; If cases are absent, THEN the use of prepositions is extensive, and vice versa;; IF order is rigid, THEN the use of prepositions is extensive, and vice versa. : IF constituent order is flexible, THEN cases are present, and vice versa; ; IF cases are present, THEN the use of prepositions is sparse, and vice versa; ; IF order is flexible, THEN the use of prepositions is sparse, and vice versa.</t>
+          <t>There are correlations between following parameters: VO word order, Non-tensedness, Non-casedness, WITH-Construction, Non-Absolute Converb. Standardized IF VO, THEN Non-tensedness, Non-casedness, WITH-Construction, and Non-Absolute Converb. IF Non-tensedness, THEN VO, Non-casedness, WITH-Construction, and Non-Absolute Converb. IF Non-casedness, THEN VO, Non-tensedness, WITH-Construction, and Non-Absolute Converb. IF AND-construction, THEN VO, Non-tensedness, Non-casedness, and Non-Absolute Converb. IF Non-Absolute Converb, THEN VO, Non-tensedness, Non-casedness, and WITH-Construction.</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>1.287232651060978</v>
+        <v>1.120180967718326</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1583,21 +1583,21 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>0095aka</t>
+          <t>0230bka</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>N-Adp &amp; (Adj-N | Rel-N) &gt; Dem-N</t>
+          <t>no case &gt; Adp-N</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>IF there are postpositions, THEN (IF adjectives precede nouns or relatives precede nouns, THEN demonstratives preced nouns and numerals precede nouns) and (IF demonstratives precede nouns or numerals precede nouns, THEN genitives precede nouns).</t>
+          <t>IF constituent order is rigid, THEN cases are absent, and vice versa; ; If cases are absent, THEN the use of prepositions is extensive, and vice versa;; IF order is rigid, THEN the use of prepositions is extensive, and vice versa. : IF constituent order is flexible, THEN cases are present, and vice versa; ; IF cases are present, THEN the use of prepositions is sparse, and vice versa; ; IF order is flexible, THEN the use of prepositions is sparse, and vice versa.</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>1.477393443877387</v>
+        <v>1.093796493909089</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1608,21 +1608,21 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>0517ka</t>
+          <t>0107cka</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>gender (1) &gt; gender (2 &amp;| 3)</t>
+          <t>VO &gt; N-Gen</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>If a language has gender distinctions in the 1st person, it always has gender distinctions in the 2nd or 3rd person, or in both.</t>
+          <t>Nominal modifiers (such as relative, adjectival, and attributive expressions) follow nouns in VO languages and precede nouns in OV languages</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>2.31003226870066</v>
+        <v>1.420083985458123</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1633,21 +1633,21 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>0513ka</t>
+          <t>0176ka</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>gender &gt; number</t>
+          <t>N-Gen &gt; N-Rel</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Universal 36. If a language has the category of gender, it always has the category of number.</t>
+          <t>If the genitive follows the noun, then the relative clause follows the noun.</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>0.8160835527307344</v>
+        <v>1.836018488718082</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1658,21 +1658,21 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>0107cka</t>
+          <t>1027aka</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>VO &gt; N-Gen</t>
+          <t>VO -&gt; no morph tense | no  case</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Nominal modifiers (such as relative, adjectival, and attributive expressions) follow nouns in VO languages and precede nouns in OV languages</t>
+          <t>There are correlations between following parameters: VO word order, Non-tensedness, Non-casedness, WITH-Construction, Non-Absolute Converb. Standardized IF VO, THEN Non-tensedness, Non-casedness, WITH-Construction, and Non-Absolute Converb. IF Non-tensedness, THEN VO, Non-casedness, WITH-Construction, and Non-Absolute Converb. IF Non-casedness, THEN VO, Non-tensedness, WITH-Construction, and Non-Absolute Converb. IF AND-construction, THEN VO, Non-tensedness, Non-casedness, and Non-Absolute Converb. IF Non-Absolute Converb, THEN VO, Non-tensedness, Non-casedness, and WITH-Construction.</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>1.412549422776825</v>
+        <v>1.460432226896094</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1683,21 +1683,21 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>0015aka</t>
+          <t>1741ka</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>OV &gt; V-Mod</t>
+          <t>Gen prefix &gt; verbal prefixes</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Verbal modifiers like those for negation, causation, and reflexive or reciprocal are placed after verb roots in OV languages and before verb roots in VO languages.</t>
+          <t>There is more prefixing on verb than on noun. If a language has any prefixes on noun, it will also have prefixes on verb with considerably more than chance frequency.</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>1.274069053984944</v>
+        <v>1.905343268029184</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1708,21 +1708,21 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>0087ka</t>
+          <t>1586ka</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Adp-N &amp; N-Dem &gt; N-Rel</t>
+          <t>poss head-marked &gt; opp alien-inalien poss</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>IF a language has Prep word order, then if the demonstrative follows the noun, the relative clause follows the noun.</t>
+          <t>An opposition of "alienable" and "inalienable" possession is almost inevitable in languages where possession is regularly head-marked. The alienable-inalienable opposition is almost never signaled by dependent-marked morphology.</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>2.180597906971648</v>
+        <v>0.9642790964745299</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -1733,21 +1733,21 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>1431mka</t>
+          <t>0513ka</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>less case &gt; more tense</t>
+          <t>gender &gt; number</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>The more developed a case system is, the less is its system of verbal tenses.</t>
+          <t>Universal 36. If a language has the category of gender, it always has the category of number.</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>-0.6442960570923952</v>
+        <v>0.8029533541850679</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -1758,21 +1758,21 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>0074ka</t>
+          <t>0107aka</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Adp-N &amp; N-Num &gt; N-Adj</t>
+          <t>VO &gt; N-Rel</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>If a language has Prep word order, then if the numeral follows the noun, the adjective follows the noun.</t>
+          <t>Nominal modifiers (such as relative, adjectival, and attributive expressions) follow nouns in VO languages and precede nouns in OV languages</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>1.212197094715449</v>
+        <v>1.374293838557867</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1783,21 +1783,21 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>1027aka</t>
+          <t>0125ka</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>VO -&gt; no morph tense | no  case</t>
+          <t>SOV &amp; Det-N &gt; N-Adp</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>There are correlations between following parameters: VO word order, Non-tensedness, Non-casedness, WITH-Construction, Non-Absolute Converb. Standardized IF VO, THEN Non-tensedness, Non-casedness, WITH-Construction, and Non-Absolute Converb. IF Non-tensedness, THEN VO, Non-casedness, WITH-Construction, and Non-Absolute Converb. IF Non-casedness, THEN VO, Non-tensedness, WITH-Construction, and Non-Absolute Converb. IF AND-construction, THEN VO, Non-tensedness, Non-casedness, and Non-Absolute Converb. IF Non-Absolute Converb, THEN VO, Non-tensedness, Non-casedness, and WITH-Construction.</t>
+          <t>If a language has both SOV in a full sentence and determining N+determined N in a Noun Phrase, then it has at least some postpositions, which historically come either from verbs (ex. Bengali), or from nouns (ex. Mande languages (W. Africa)).</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>1.424790430069664</v>
+        <v>1.444144182948785</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1808,21 +1808,21 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>0125ka</t>
+          <t>1114ka</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>SOV &amp; Det-N &gt; N-Adp</t>
+          <t>VO &gt; Comp-S</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>If a language has both SOV in a full sentence and determining N+determined N in a Noun Phrase, then it has at least some postpositions, which historically come either from verbs (ex. Bengali), or from nouns (ex. Mande languages (W. Africa)).</t>
+          <t>VO languages are exceptionlessly Comp-initial. OV languages exemplify both final complementizers and initial complementizers.</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>1.518727899166531</v>
+        <v>1.200667430958548</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1833,21 +1833,21 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>0107aka</t>
+          <t>0087ka</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>VO &gt; N-Rel</t>
+          <t>Adp-N &amp; N-Dem &gt; N-Rel</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Nominal modifiers (such as relative, adjectival, and attributive expressions) follow nouns in VO languages and precede nouns in OV languages</t>
+          <t>IF a language has Prep word order, then if the demonstrative follows the noun, the relative clause follows the noun.</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>1.372169819140258</v>
+        <v>2.029631662382088</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1858,21 +1858,21 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>0176ka</t>
+          <t>0423ka</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>N-Gen &gt; N-Rel</t>
+          <t>Adp-N &amp; no SOV &gt; N-Rel</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>If the genitive follows the noun, then the relative clause follows the noun.</t>
+          <t>If a language has Prep word order, then if the verb position is not SOV, the relative clause follows the noun.</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>1.609040846358095</v>
+        <v>1.487332637489372</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1883,21 +1883,21 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>0423ka</t>
+          <t>1431mka</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Adp-N &amp; no SOV &gt; N-Rel</t>
+          <t>less case &gt; more tense</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>If a language has Prep word order, then if the verb position is not SOV, the relative clause follows the noun.</t>
+          <t>The more developed a case system is, the less is its system of verbal tenses.</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>1.587761166121661</v>
+        <v>-0.6922248006702326</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1908,48 +1908,23 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>1114ka</t>
+          <t>0175ka</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>VO &gt; Comp-S</t>
+          <t>Adp-N &amp; N-Gen &gt; N-Rel</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>VO languages are exceptionlessly Comp-initial. OV languages exemplify both final complementizers and initial complementizers.</t>
+          <t>If a language has Prep word order, then if the genitive follows the noun, the relative clause follows the noun.</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>1.16047995573335</v>
+        <v>1.66594161299483</v>
       </c>
       <c r="E60" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>0175ka</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>Adp-N &amp; N-Gen &gt; N-Rel</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>If a language has Prep word order, then if the genitive follows the noun, the relative clause follows the noun.</t>
-        </is>
-      </c>
-      <c r="D61" t="n">
-        <v>1.700500960391001</v>
-      </c>
-      <c r="E61" t="inlineStr">
         <is>
           <t>Both</t>
         </is>

</xml_diff>